<commit_message>
Parity colours address-based (fix bottom-amber after template re-save) + drop remarks patch
Root cause of the "mysterious amber at the bottom" (and stray borders on even
races): applyRaceParityHeaderStyle + setRemarksAlignmentXlsx hardcoded style
indices (37/38, 11/17), which Excel renumbers on every template re-save — so the
edits landed on the wrong (bottom) cells.

- applyRaceParityHeaderStyle now resolves row-1 styles BY ADDRESS (A1 = title,
  D1 = result/time) and re-points ONLY row-1 cells (r="X1"). Robust to template
  re-saves; nothing outside row 1 is ever touched.
- Dropped the remarks-alignment patch (also index-based) from the export + draw
  pipelines — borders/alignment are now handled in the (operator-edited)
  race-template.xlsx.
- Bundle the updated race-template.xlsx (operator's border fixes).
- Smoke test made template-agnostic (asserts A1 re-pointed to an appended clone).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rdms/templates/race-template.xlsx
+++ b/rdms/templates/race-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gautamahou/Library/CloudStorage/GoogleDrive-no_reply@dragonboat.org.hk/My Drive/SDBA Events/Events/2026WU/01 Input_Draw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gautamahou/Projects/git/sdbafinishing.github.io/rdms/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA99E327-9202-7C40-A10F-B9C38CEE50A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0803D27-EC39-1B44-9C30-3CC334726CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="21360" xr2:uid="{01510F48-7312-BC41-A2B0-D047B7B26968}"/>
   </bookViews>
@@ -19,206 +19,20 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$I$19</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="32">
   <si>
-    <r>
-      <t xml:space="preserve">BOAT 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>船號</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Team Name
- </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>隊伍名稱</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Code
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>編號</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">成績   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Result</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">備註
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Arial Unicode MS"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>Remarks</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Time </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>時間</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Place 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>名次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Score
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>分數</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Total Score
- </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>總分數</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Total Place
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="新細明體"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t>總名次</t>
-    </r>
-  </si>
-  <si>
     <t>Chief Judge Signature :</t>
   </si>
   <si>
     <t>Signature Time :</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">裁判簽署 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="Arial Unicode MS"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">簽署時間 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="Arial Unicode MS"/>
-        <family val="1"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-  </si>
-  <si>
     <t>Race No. 1 --- 男子組 標準龍 初賽  Men's Division Standard Boat - Heats - 場次 Race 1</t>
-    <phoneticPr fontId="33" type="noConversion"/>
+    <phoneticPr fontId="22" type="noConversion"/>
   </si>
   <si>
     <t>8:30</t>
@@ -272,7 +86,51 @@
     <t xml:space="preserve">*Private Steersman
 各初賽第1至4名晉級至「盃複賽」，其餘獲邀參加「碟決賽」。
 Teams in 1st Place to 4th Place will advance to the “Cup Semi-finals", the rest will advance to the " Plate Finals". </t>
-    <phoneticPr fontId="33" type="noConversion"/>
+    <phoneticPr fontId="22" type="noConversion"/>
+  </si>
+  <si>
+    <t>BOAT 
+船號</t>
+  </si>
+  <si>
+    <t>Team Name
+ 隊伍名稱</t>
+  </si>
+  <si>
+    <t>Code
+編號</t>
+  </si>
+  <si>
+    <t>成績   Result</t>
+  </si>
+  <si>
+    <t>備註
+Remarks</t>
+  </si>
+  <si>
+    <t>Time 時間</t>
+  </si>
+  <si>
+    <t>Place 
+名次</t>
+  </si>
+  <si>
+    <t>Score
+分數</t>
+  </si>
+  <si>
+    <t>Total Score
+ 總分數</t>
+  </si>
+  <si>
+    <t>Total Place
+總名次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">裁判簽署 : </t>
+  </si>
+  <si>
+    <t xml:space="preserve">簽署時間 : </t>
   </si>
 </sst>
 </file>
@@ -280,9 +138,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="188" formatCode="0.00_ "/>
+    <numFmt numFmtId="164" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <name val="新細明體"/>
@@ -420,85 +278,54 @@
       <charset val="136"/>
     </font>
     <font>
-      <sz val="16"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <name val="Arial Unicode MS"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial Unicode MS"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Arial Unicode MS"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <name val="Arial Unicode MS"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <name val="新細明體"/>
       <family val="1"/>
       <charset val="136"/>
     </font>
     <font>
-      <sz val="16"/>
-      <name val="Arial Unicode MS"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="20"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="新細明體"/>
-      <family val="1"/>
-      <charset val="136"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="新細明體"/>
       <family val="1"/>
       <charset val="136"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="24">
@@ -1180,7 +1007,7 @@
     <xf numFmtId="0" fontId="13" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="7" applyNumberFormat="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="7" applyNumberFormat="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="20" borderId="8" applyNumberFormat="0" applyProtection="0">
@@ -1323,135 +1150,126 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="23" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="188" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="188" fontId="25" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="85">
@@ -1909,363 +1727,347 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED9A5213-6DAB-2B4E-B509-98B58017F784}">
-  <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="36" defaultRowHeight="22"/>
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="36" defaultRowHeight="20"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="70.1640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.5" style="2" customWidth="1"/>
-    <col min="5" max="5" width="7.1640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.1640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="9.83203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="7.1640625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="7.5" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="36" style="2"/>
+    <col min="1" max="1" width="9" style="39" customWidth="1"/>
+    <col min="2" max="2" width="70.1640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="9" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="3" customWidth="1"/>
+    <col min="5" max="5" width="7.1640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="8.1640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="7.1640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="7.5" style="3" customWidth="1"/>
+    <col min="10" max="16384" width="36" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="37.25" customHeight="1">
-      <c r="A1" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9" ht="19.5" customHeight="1">
-      <c r="A2" s="39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="40" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="39" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="41" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="42" t="s">
-        <v>4</v>
+      <c r="A2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="7" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="59.25" customHeight="1">
-      <c r="A3" s="39"/>
-      <c r="B3" s="40"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="42"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="7"/>
     </row>
     <row r="4" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A4" s="6">
+      <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="11"/>
+      <c r="B4" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="16"/>
     </row>
     <row r="5" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A5" s="12">
+      <c r="A5" s="17">
         <v>2</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="17"/>
+      <c r="B5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A6" s="12">
+      <c r="A6" s="17">
         <v>3</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I6" s="17"/>
+      <c r="B6" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" s="22"/>
     </row>
     <row r="7" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A7" s="12">
+      <c r="A7" s="17">
         <v>4</v>
       </c>
-      <c r="B7" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I7" s="17"/>
+      <c r="B7" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="22"/>
     </row>
     <row r="8" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A8" s="12">
+      <c r="A8" s="17">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="17"/>
+      <c r="B8" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="22"/>
     </row>
     <row r="9" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A9" s="12">
-        <v>6</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I9" s="17"/>
+      <c r="A9" s="17">
+        <v>6</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="22"/>
     </row>
     <row r="10" spans="1:9" ht="22.25" customHeight="1">
-      <c r="A10" s="12">
+      <c r="A10" s="17">
         <v>7</v>
       </c>
-      <c r="B10" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="15" t="s">
+      <c r="B10" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I10" s="17"/>
+      <c r="D10" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="22"/>
     </row>
     <row r="11" spans="1:9" ht="9.5" customHeight="1">
-      <c r="A11" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
-      <c r="I11" s="30"/>
+      <c r="A11" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="26"/>
     </row>
     <row r="12" spans="1:9" ht="9.5" customHeight="1">
-      <c r="A12" s="31"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="33"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="29"/>
     </row>
     <row r="13" spans="1:9" ht="9.5" customHeight="1">
-      <c r="A13" s="31"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="33"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="29"/>
     </row>
     <row r="14" spans="1:9" ht="37.5" customHeight="1" thickBot="1">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="36"/>
+      <c r="A14" s="30"/>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="32"/>
     </row>
     <row r="15" spans="1:9" ht="21.5" customHeight="1">
-      <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
     </row>
     <row r="16" spans="1:9" ht="21.5" customHeight="1">
-      <c r="A16" s="19"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
     </row>
     <row r="17" spans="1:9" ht="32" customHeight="1">
-      <c r="A17" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
+      <c r="A17" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
     </row>
     <row r="18" spans="1:9" ht="32" customHeight="1">
-      <c r="A18" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
+      <c r="A18" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="37"/>
+      <c r="D18" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
     </row>
     <row r="19" spans="1:9" ht="32" customHeight="1"/>
-    <row r="21" spans="1:9">
-      <c r="A21" s="26"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="8">
@@ -2278,11 +2080,11 @@
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="I2:I3"/>
   </mergeCells>
-  <phoneticPr fontId="33" type="noConversion"/>
+  <phoneticPr fontId="22" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.51180555555555551"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter alignWithMargins="0">
-    <oddHeader>&amp;C&amp;"Arial Unicode MS,標準"Stanley Dragon Boat Warm Up 250
+    <oddHeader>&amp;C&amp;"Arial,Regular"Stanley Dragon Boat Warm Up 250
 赤柱龍舟熱身賽 250</oddHeader>
   </headerFooter>
 </worksheet>

</xml_diff>